<commit_message>
Massive overhaul of styling and diverse bug fixes
- changed popups
- fixed descriptions of layers
- fixed missing indicator labels
- fixed updating logic of new indicators and how they get added to the tool
- added icons for selected layers in the active layer tab
- added outlines for polygons in color mode
- removed some unnecessary commentary and bloat
</commit_message>
<xml_diff>
--- a/scripts/Indicators_Inside_Tool.xlsx
+++ b/scripts/Indicators_Inside_Tool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Martin\Desktop\June_12_Update_ADM1_2_3_New_SHP\Political_VUL_Change\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Martin\Documents\GitHub\LB_DEV\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E91389D5-8370-4E1F-ABFE-13E8D251B82E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB0FF27C-9044-4841-915C-A9710FD46FCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9BB32CAF-FA07-415F-97C1-8C7F5920FABD}"/>
+    <workbookView xWindow="12" yWindow="12" windowWidth="23016" windowHeight="12336" xr2:uid="{9BB32CAF-FA07-415F-97C1-8C7F5920FABD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="233">
   <si>
     <t>PV1</t>
   </si>
@@ -266,18 +266,12 @@
     <t>S9</t>
   </si>
   <si>
-    <t>Demographic Tension / Stress</t>
-  </si>
-  <si>
     <t>T17</t>
   </si>
   <si>
     <t>Demographic Shock Factor</t>
   </si>
   <si>
-    <t>Climate and Environmental Risk</t>
-  </si>
-  <si>
     <t>E1</t>
   </si>
   <si>
@@ -626,17 +620,249 @@
     <t>Additional kg per day generated in a particular locality</t>
   </si>
   <si>
-    <t>% change in number of consecutive hot days per year;</t>
-  </si>
-  <si>
     <t>% change in number of forest fires per district;</t>
+  </si>
+  <si>
+    <t>To what extent is internal displacement leading to demographic tension?</t>
+  </si>
+  <si>
+    <t>E4</t>
+  </si>
+  <si>
+    <t>E5</t>
+  </si>
+  <si>
+    <t>E6</t>
+  </si>
+  <si>
+    <t>Consecutive Dry Days</t>
+  </si>
+  <si>
+    <t>Consecutive Wet Days</t>
+  </si>
+  <si>
+    <t>Days with at least 10 mm rainfall</t>
+  </si>
+  <si>
+    <t>Days with at least 20 mm rainfall</t>
+  </si>
+  <si>
+    <t>Very Hot Days (Tmax &gt; 35°C)</t>
+  </si>
+  <si>
+    <t>Hot days (Tmax &gt; 30°C)</t>
+  </si>
+  <si>
+    <t>E7</t>
+  </si>
+  <si>
+    <t>E8</t>
+  </si>
+  <si>
+    <t>Climate Risk</t>
+  </si>
+  <si>
+    <t>How is the quality of education perceived among the population?</t>
+  </si>
+  <si>
+    <t>How is the quality of healthcare services perceived among the population?</t>
+  </si>
+  <si>
+    <t>How often do tensions around electricity manifest in incidents?</t>
+  </si>
+  <si>
+    <t>How often do tensions around private generators manifest in incidents?</t>
+  </si>
+  <si>
+    <t>How often do tensions around health manifest in incidents?</t>
+  </si>
+  <si>
+    <t>How often do tensions around education manifest in incidents?</t>
+  </si>
+  <si>
+    <t>How often do tensions around civil defense manifest in incidents?</t>
+  </si>
+  <si>
+    <t>% of respondents rating the quality of education services as poor or very poor</t>
+  </si>
+  <si>
+    <t>% of respondents rating the quality of healthcare services as poor or very poor</t>
+  </si>
+  <si>
+    <t>number of tension incidents around electricity services and provision</t>
+  </si>
+  <si>
+    <t>number of tension incidents around private generator services and provision</t>
+  </si>
+  <si>
+    <t>number of tension incidents around private health services and provision</t>
+  </si>
+  <si>
+    <t>number of tension incidents around education services and provision</t>
+  </si>
+  <si>
+    <t>number of tension incidents around civil defense services</t>
+  </si>
+  <si>
+    <t>E9</t>
+  </si>
+  <si>
+    <t>How many consecutive days without precipitation</t>
+  </si>
+  <si>
+    <t>Consecutive dry days (CDD) is a climate index defined as the maximum number of continuous days in a specific period where precipitation is below a defined threshold, usually less than 1 mm per day</t>
+  </si>
+  <si>
+    <t>Days with temperatures above 30 °C</t>
+  </si>
+  <si>
+    <t>Days with temperatures above 35 °C</t>
+  </si>
+  <si>
+    <t>Consecutive wet days refer to an unbroken sequence of days where each day records a measurable amount of precipitation meeting or exceeding a specific threshold, typically 1 millimeter</t>
+  </si>
+  <si>
+    <t>Days with at least 10mm rainfall</t>
+  </si>
+  <si>
+    <t>Days with at least 20mm rainfall</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Days with temperatures above 35 °C are commonly classified in climatology and meteorology as </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>extreme summer days</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> or days contributing to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>extreme heat</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>heat stress</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> indices</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Days with temperatures above 30 °C are commonly classified in climatology and meteorology as </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>extreme summer days</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> or days contributing to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>extreme heat</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>heat stress</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> indices</t>
+    </r>
+  </si>
+  <si>
+    <t>A day with at least 10mm of rainfall is officially classified in meteorology as a day of moderate-to-heavy precipitation or a heavy precipitation day</t>
+  </si>
+  <si>
+    <t>In climatology, the phrase "days with at least 20mm rainfall" refers to a standard climate index known as R20mm, which measures the frequency of very heavy precipitation days</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -651,6 +877,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -679,10 +911,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1017,21 +1250,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8ECAF9A-B5D0-4237-9E56-A4DD366B9284}">
-  <dimension ref="A1:I47"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I53"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="47" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.42578125" customWidth="1"/>
-    <col min="9" max="9" width="48.7109375" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.44140625" customWidth="1"/>
+    <col min="9" max="9" width="48.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>59</v>
       </c>
@@ -1054,13 +1287,13 @@
         <v>27</v>
       </c>
       <c r="H1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>7</v>
       </c>
@@ -1071,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E2" t="s">
         <v>30</v>
@@ -1080,16 +1313,16 @@
         <v>24</v>
       </c>
       <c r="G2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>7</v>
       </c>
@@ -1109,16 +1342,16 @@
         <v>24</v>
       </c>
       <c r="G3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>7</v>
       </c>
@@ -1129,7 +1362,7 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E4" t="s">
         <v>30</v>
@@ -1138,16 +1371,16 @@
         <v>24</v>
       </c>
       <c r="G4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>7</v>
       </c>
@@ -1158,7 +1391,7 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E5" t="s">
         <v>30</v>
@@ -1167,16 +1400,16 @@
         <v>24</v>
       </c>
       <c r="G5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>7</v>
       </c>
@@ -1187,7 +1420,7 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E6" t="s">
         <v>30</v>
@@ -1196,16 +1429,16 @@
         <v>24</v>
       </c>
       <c r="G6" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I6" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
@@ -1216,7 +1449,7 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E7" t="s">
         <v>30</v>
@@ -1225,16 +1458,16 @@
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="I7" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1245,7 +1478,7 @@
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E8" t="s">
         <v>30</v>
@@ -1254,16 +1487,16 @@
         <v>24</v>
       </c>
       <c r="G8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H8" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I8" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -1274,7 +1507,7 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E9" t="s">
         <v>30</v>
@@ -1283,16 +1516,16 @@
         <v>24</v>
       </c>
       <c r="G9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I9" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>7</v>
       </c>
@@ -1300,97 +1533,97 @@
         <v>58</v>
       </c>
       <c r="C10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" t="s">
+        <v>86</v>
+      </c>
+      <c r="G10" t="s">
+        <v>88</v>
+      </c>
+      <c r="H10" t="s">
+        <v>194</v>
+      </c>
+      <c r="I10" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" t="s">
         <v>9</v>
       </c>
-      <c r="D10" t="s">
-        <v>178</v>
-      </c>
-      <c r="E10" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="D11" t="s">
+        <v>176</v>
+      </c>
+      <c r="E11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" t="s">
         <v>25</v>
-      </c>
-      <c r="G10" t="s">
-        <v>29</v>
-      </c>
-      <c r="H10" t="s">
-        <v>137</v>
-      </c>
-      <c r="I10" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>8</v>
-      </c>
-      <c r="B11" t="s">
-        <v>86</v>
-      </c>
-      <c r="C11" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>30</v>
-      </c>
-      <c r="F11" t="s">
-        <v>26</v>
       </c>
       <c r="G11" t="s">
         <v>29</v>
       </c>
       <c r="H11" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="I11" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D12" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E12" t="s">
         <v>30</v>
       </c>
       <c r="F12" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G12" t="s">
-        <v>95</v>
+        <v>29</v>
       </c>
       <c r="H12" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="I12" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C13" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>179</v>
+        <v>13</v>
       </c>
       <c r="E13" t="s">
         <v>30</v>
@@ -1399,27 +1632,27 @@
         <v>24</v>
       </c>
       <c r="G13" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H13" t="s">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="I13" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D14" t="s">
-        <v>16</v>
+        <v>177</v>
       </c>
       <c r="E14" t="s">
         <v>30</v>
@@ -1428,27 +1661,27 @@
         <v>24</v>
       </c>
       <c r="G14" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H14" t="s">
+        <v>115</v>
+      </c>
+      <c r="I14" t="s">
         <v>116</v>
       </c>
-      <c r="I14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C15" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D15" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E15" t="s">
         <v>30</v>
@@ -1457,27 +1690,27 @@
         <v>24</v>
       </c>
       <c r="G15" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H15" t="s">
-        <v>143</v>
+        <v>114</v>
       </c>
       <c r="I15" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>8</v>
       </c>
       <c r="B16" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C16" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D16" t="s">
-        <v>180</v>
+        <v>18</v>
       </c>
       <c r="E16" t="s">
         <v>30</v>
@@ -1486,27 +1719,27 @@
         <v>24</v>
       </c>
       <c r="G16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H16" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="I16" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>8</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C17" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="D17" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="E17" t="s">
         <v>30</v>
@@ -1515,74 +1748,74 @@
         <v>24</v>
       </c>
       <c r="G17" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H17" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="I17" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
+        <v>8</v>
+      </c>
+      <c r="B18" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" t="s">
+        <v>179</v>
+      </c>
+      <c r="E18" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" t="s">
+        <v>24</v>
+      </c>
+      <c r="G18" t="s">
+        <v>93</v>
+      </c>
+      <c r="H18" t="s">
+        <v>143</v>
+      </c>
+      <c r="I18" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19">
         <v>1</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B19" t="s">
         <v>32</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C19" t="s">
+        <v>180</v>
+      </c>
+      <c r="D19" t="s">
+        <v>85</v>
+      </c>
+      <c r="E19" t="s">
+        <v>30</v>
+      </c>
+      <c r="F19" t="s">
+        <v>86</v>
+      </c>
+      <c r="G19" t="s">
+        <v>28</v>
+      </c>
+      <c r="H19" t="s">
+        <v>181</v>
+      </c>
+      <c r="I19" t="s">
         <v>182</v>
       </c>
-      <c r="D18" t="s">
-        <v>87</v>
-      </c>
-      <c r="E18" t="s">
-        <v>30</v>
-      </c>
-      <c r="F18" t="s">
-        <v>88</v>
-      </c>
-      <c r="G18" t="s">
-        <v>28</v>
-      </c>
-      <c r="H18" t="s">
-        <v>183</v>
-      </c>
-      <c r="I18" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>2</v>
-      </c>
-      <c r="B19" t="s">
-        <v>33</v>
-      </c>
-      <c r="C19" t="s">
-        <v>34</v>
-      </c>
-      <c r="D19" t="s">
-        <v>43</v>
-      </c>
-      <c r="E19" t="s">
-        <v>30</v>
-      </c>
-      <c r="F19" t="s">
-        <v>91</v>
-      </c>
-      <c r="G19" t="s">
-        <v>29</v>
-      </c>
-      <c r="H19" t="s">
-        <v>110</v>
-      </c>
-      <c r="I19" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2</v>
       </c>
@@ -1590,28 +1823,28 @@
         <v>33</v>
       </c>
       <c r="C20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E20" t="s">
         <v>30</v>
       </c>
       <c r="F20" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G20" t="s">
         <v>29</v>
       </c>
       <c r="H20" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="I20" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2</v>
       </c>
@@ -1619,28 +1852,28 @@
         <v>33</v>
       </c>
       <c r="C21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E21" t="s">
         <v>30</v>
       </c>
       <c r="F21" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G21" t="s">
         <v>29</v>
       </c>
       <c r="H21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I21" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2</v>
       </c>
@@ -1648,28 +1881,28 @@
         <v>33</v>
       </c>
       <c r="C22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E22" t="s">
         <v>30</v>
       </c>
       <c r="F22" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="G22" t="s">
         <v>29</v>
       </c>
       <c r="H22" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="I22" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2</v>
       </c>
@@ -1677,28 +1910,28 @@
         <v>33</v>
       </c>
       <c r="C23" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E23" t="s">
         <v>30</v>
       </c>
       <c r="F23" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
       <c r="G23" t="s">
-        <v>95</v>
+        <v>29</v>
       </c>
       <c r="H23" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="I23" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2</v>
       </c>
@@ -1706,10 +1939,10 @@
         <v>33</v>
       </c>
       <c r="C24" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E24" t="s">
         <v>30</v>
@@ -1718,45 +1951,45 @@
         <v>24</v>
       </c>
       <c r="G24" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I24" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B25" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C25" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="D25" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E25" t="s">
-        <v>96</v>
+        <v>30</v>
       </c>
       <c r="F25" t="s">
-        <v>97</v>
+        <v>24</v>
       </c>
       <c r="G25" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="H25" t="s">
-        <v>169</v>
+        <v>115</v>
       </c>
       <c r="I25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>3</v>
       </c>
@@ -1764,28 +1997,28 @@
         <v>39</v>
       </c>
       <c r="C26" t="s">
-        <v>185</v>
+        <v>40</v>
       </c>
       <c r="D26" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="E26" t="s">
-        <v>30</v>
+        <v>94</v>
       </c>
       <c r="F26" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="G26" t="s">
-        <v>28</v>
+        <v>96</v>
       </c>
       <c r="H26" t="s">
-        <v>186</v>
+        <v>167</v>
       </c>
       <c r="I26" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>3</v>
       </c>
@@ -1793,57 +2026,57 @@
         <v>39</v>
       </c>
       <c r="C27" t="s">
+        <v>183</v>
+      </c>
+      <c r="D27" t="s">
+        <v>49</v>
+      </c>
+      <c r="E27" t="s">
+        <v>30</v>
+      </c>
+      <c r="F27" t="s">
+        <v>86</v>
+      </c>
+      <c r="G27" t="s">
+        <v>28</v>
+      </c>
+      <c r="H27" t="s">
+        <v>184</v>
+      </c>
+      <c r="I27" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>3</v>
+      </c>
+      <c r="B28" t="s">
+        <v>39</v>
+      </c>
+      <c r="C28" t="s">
+        <v>186</v>
+      </c>
+      <c r="D28" t="s">
+        <v>187</v>
+      </c>
+      <c r="E28" t="s">
+        <v>30</v>
+      </c>
+      <c r="F28" t="s">
+        <v>97</v>
+      </c>
+      <c r="G28" t="s">
+        <v>189</v>
+      </c>
+      <c r="H28" t="s">
+        <v>185</v>
+      </c>
+      <c r="I28" t="s">
         <v>188</v>
       </c>
-      <c r="D27" t="s">
-        <v>189</v>
-      </c>
-      <c r="E27" t="s">
-        <v>30</v>
-      </c>
-      <c r="F27" t="s">
-        <v>99</v>
-      </c>
-      <c r="G27" t="s">
-        <v>191</v>
-      </c>
-      <c r="H27" t="s">
-        <v>187</v>
-      </c>
-      <c r="I27" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>4</v>
-      </c>
-      <c r="B28" t="s">
-        <v>42</v>
-      </c>
-      <c r="C28" t="s">
-        <v>68</v>
-      </c>
-      <c r="D28" t="s">
-        <v>50</v>
-      </c>
-      <c r="E28" t="s">
-        <v>30</v>
-      </c>
-      <c r="F28" t="s">
-        <v>100</v>
-      </c>
-      <c r="G28" t="s">
-        <v>29</v>
-      </c>
-      <c r="H28" t="s">
-        <v>119</v>
-      </c>
-      <c r="I28" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>4</v>
       </c>
@@ -1851,28 +2084,28 @@
         <v>42</v>
       </c>
       <c r="C29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D29" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E29" t="s">
         <v>30</v>
       </c>
       <c r="F29" t="s">
-        <v>24</v>
+        <v>98</v>
       </c>
       <c r="G29" t="s">
-        <v>95</v>
+        <v>29</v>
       </c>
       <c r="H29" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
       <c r="I29" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>4</v>
       </c>
@@ -1880,10 +2113,10 @@
         <v>42</v>
       </c>
       <c r="C30" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D30" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E30" t="s">
         <v>30</v>
@@ -1892,16 +2125,16 @@
         <v>24</v>
       </c>
       <c r="G30" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H30" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="I30" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>4</v>
       </c>
@@ -1909,10 +2142,10 @@
         <v>42</v>
       </c>
       <c r="C31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D31" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E31" t="s">
         <v>30</v>
@@ -1921,16 +2154,16 @@
         <v>24</v>
       </c>
       <c r="G31" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H31" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I31" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>4</v>
       </c>
@@ -1938,10 +2171,10 @@
         <v>42</v>
       </c>
       <c r="C32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D32" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E32" t="s">
         <v>30</v>
@@ -1950,16 +2183,16 @@
         <v>24</v>
       </c>
       <c r="G32" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H32" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="I32" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>4</v>
       </c>
@@ -1967,10 +2200,10 @@
         <v>42</v>
       </c>
       <c r="C33" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D33" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E33" t="s">
         <v>30</v>
@@ -1979,16 +2212,16 @@
         <v>24</v>
       </c>
       <c r="G33" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H33" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="I33" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>4</v>
       </c>
@@ -1996,10 +2229,10 @@
         <v>42</v>
       </c>
       <c r="C34" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E34" t="s">
         <v>30</v>
@@ -2008,16 +2241,16 @@
         <v>24</v>
       </c>
       <c r="G34" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H34" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="I34" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>4</v>
       </c>
@@ -2025,10 +2258,10 @@
         <v>42</v>
       </c>
       <c r="C35" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D35" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E35" t="s">
         <v>30</v>
@@ -2037,16 +2270,16 @@
         <v>24</v>
       </c>
       <c r="G35" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H35" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="I35" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>4</v>
       </c>
@@ -2054,28 +2287,28 @@
         <v>42</v>
       </c>
       <c r="C36" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="D36" t="s">
-        <v>193</v>
+        <v>54</v>
       </c>
       <c r="E36" t="s">
         <v>30</v>
       </c>
       <c r="F36" t="s">
-        <v>101</v>
+        <v>24</v>
       </c>
       <c r="G36" t="s">
-        <v>192</v>
+        <v>93</v>
       </c>
       <c r="H36" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="I36" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>4</v>
       </c>
@@ -2083,22 +2316,28 @@
         <v>42</v>
       </c>
       <c r="C37" t="s">
-        <v>163</v>
+        <v>83</v>
       </c>
       <c r="D37" t="s">
-        <v>60</v>
+        <v>191</v>
       </c>
       <c r="E37" t="s">
         <v>30</v>
       </c>
       <c r="F37" t="s">
-        <v>24</v>
+        <v>99</v>
       </c>
       <c r="G37" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+      <c r="H37" t="s">
+        <v>159</v>
+      </c>
+      <c r="I37" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>4</v>
       </c>
@@ -2106,10 +2345,10 @@
         <v>42</v>
       </c>
       <c r="C38" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D38" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E38" t="s">
         <v>30</v>
@@ -2118,10 +2357,16 @@
         <v>24</v>
       </c>
       <c r="G38" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+      <c r="H38" t="s">
+        <v>159</v>
+      </c>
+      <c r="I38" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>4</v>
       </c>
@@ -2129,22 +2374,28 @@
         <v>42</v>
       </c>
       <c r="C39" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D39" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E39" t="s">
         <v>30</v>
       </c>
       <c r="F39" t="s">
-        <v>104</v>
+        <v>24</v>
       </c>
       <c r="G39" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+      <c r="H39" t="s">
+        <v>207</v>
+      </c>
+      <c r="I39" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>4</v>
       </c>
@@ -2152,22 +2403,28 @@
         <v>42</v>
       </c>
       <c r="C40" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D40" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E40" t="s">
         <v>30</v>
       </c>
       <c r="F40" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G40" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H40" t="s">
+        <v>208</v>
+      </c>
+      <c r="I40" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>4</v>
       </c>
@@ -2175,22 +2432,28 @@
         <v>42</v>
       </c>
       <c r="C41" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="D41" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E41" t="s">
         <v>30</v>
       </c>
       <c r="F41" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G41" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H41" t="s">
+        <v>209</v>
+      </c>
+      <c r="I41" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>4</v>
       </c>
@@ -2198,22 +2461,28 @@
         <v>42</v>
       </c>
       <c r="C42" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D42" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E42" t="s">
         <v>30</v>
       </c>
       <c r="F42" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="G42" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H42" t="s">
+        <v>210</v>
+      </c>
+      <c r="I42" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>4</v>
       </c>
@@ -2221,120 +2490,291 @@
         <v>42</v>
       </c>
       <c r="C43" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D43" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E43" t="s">
         <v>30</v>
       </c>
       <c r="F43" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G43" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H43" t="s">
+        <v>211</v>
+      </c>
+      <c r="I43" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B44" t="s">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="C44" t="s">
-        <v>76</v>
+        <v>166</v>
       </c>
       <c r="D44" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="E44" t="s">
         <v>30</v>
       </c>
       <c r="F44" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G44" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="H44" t="s">
+        <v>212</v>
+      </c>
+      <c r="I44" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>78</v>
+        <v>206</v>
       </c>
       <c r="C45" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D45" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E45" t="s">
         <v>30</v>
       </c>
       <c r="F45" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G45" t="s">
         <v>29</v>
       </c>
       <c r="H45" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+        <v>213</v>
+      </c>
+      <c r="I45" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>6</v>
       </c>
       <c r="B46" t="s">
+        <v>206</v>
+      </c>
+      <c r="C46" t="s">
         <v>78</v>
       </c>
-      <c r="C46" t="s">
-        <v>80</v>
-      </c>
       <c r="D46" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E46" t="s">
         <v>30</v>
       </c>
       <c r="F46" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G46" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H46" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>6</v>
       </c>
       <c r="B47" t="s">
-        <v>78</v>
+        <v>206</v>
       </c>
       <c r="C47" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D47" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E47" t="s">
         <v>30</v>
       </c>
       <c r="F47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G47" t="s">
         <v>29</v>
       </c>
       <c r="H47" t="s">
-        <v>170</v>
+        <v>168</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>6</v>
+      </c>
+      <c r="B48" t="s">
+        <v>206</v>
+      </c>
+      <c r="C48" t="s">
+        <v>195</v>
+      </c>
+      <c r="D48" t="s">
+        <v>198</v>
+      </c>
+      <c r="E48" t="s">
+        <v>30</v>
+      </c>
+      <c r="G48" t="s">
+        <v>29</v>
+      </c>
+      <c r="H48" t="s">
+        <v>222</v>
+      </c>
+      <c r="I48" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>6</v>
+      </c>
+      <c r="B49" t="s">
+        <v>206</v>
+      </c>
+      <c r="C49" t="s">
+        <v>196</v>
+      </c>
+      <c r="D49" t="s">
+        <v>199</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="G49" t="s">
+        <v>29</v>
+      </c>
+      <c r="H49" t="s">
+        <v>222</v>
+      </c>
+      <c r="I49" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>6</v>
+      </c>
+      <c r="B50" t="s">
+        <v>206</v>
+      </c>
+      <c r="C50" t="s">
+        <v>197</v>
+      </c>
+      <c r="D50" t="s">
+        <v>200</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="G50" t="s">
+        <v>29</v>
+      </c>
+      <c r="H50" t="s">
+        <v>227</v>
+      </c>
+      <c r="I50" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>6</v>
+      </c>
+      <c r="B51" t="s">
+        <v>206</v>
+      </c>
+      <c r="C51" t="s">
+        <v>204</v>
+      </c>
+      <c r="D51" t="s">
+        <v>201</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="G51" t="s">
+        <v>29</v>
+      </c>
+      <c r="H51" t="s">
+        <v>228</v>
+      </c>
+      <c r="I51" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>6</v>
+      </c>
+      <c r="B52" t="s">
+        <v>206</v>
+      </c>
+      <c r="C52" t="s">
+        <v>205</v>
+      </c>
+      <c r="D52" t="s">
+        <v>202</v>
+      </c>
+      <c r="E52" t="s">
+        <v>30</v>
+      </c>
+      <c r="G52" t="s">
+        <v>29</v>
+      </c>
+      <c r="H52" t="s">
+        <v>225</v>
+      </c>
+      <c r="I52" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>6</v>
+      </c>
+      <c r="B53" t="s">
+        <v>206</v>
+      </c>
+      <c r="C53" t="s">
+        <v>221</v>
+      </c>
+      <c r="D53" t="s">
+        <v>203</v>
+      </c>
+      <c r="E53" t="s">
+        <v>30</v>
+      </c>
+      <c r="G53" t="s">
+        <v>29</v>
+      </c>
+      <c r="H53" t="s">
+        <v>224</v>
+      </c>
+      <c r="I53" t="s">
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -2343,14 +2783,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="df1c7a3b-3e5b-458f-b25e-72cfea04893a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008E84AF0C558E1541AF7F3527107E44B2" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="29590c1f38a0215f82f617aa18ae2e52">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="df1c7a3b-3e5b-458f-b25e-72cfea04893a" xmlns:ns4="571ba4f1-bf68-41bf-beab-afb721956c8b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1509126a86945b625aae62f3004de406" ns3:_="" ns4:_="">
     <xsd:import namespace="df1c7a3b-3e5b-458f-b25e-72cfea04893a"/>
@@ -2603,7 +3035,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2612,24 +3044,15 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29F12554-73D9-44F3-9A50-857E772D550B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="df1c7a3b-3e5b-458f-b25e-72cfea04893a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="571ba4f1-bf68-41bf-beab-afb721956c8b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="df1c7a3b-3e5b-458f-b25e-72cfea04893a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D88FE89E-22A8-4DEC-97DF-98F2D295E9E0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2648,10 +3071,27 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB8AA580-F103-47C9-9131-88C699F85CBD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29F12554-73D9-44F3-9A50-857E772D550B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="df1c7a3b-3e5b-458f-b25e-72cfea04893a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="571ba4f1-bf68-41bf-beab-afb721956c8b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>